<commit_message>
Implement gas in case study
Fix wrong gas paths in ExcelWriter
</commit_message>
<xml_diff>
--- a/data/example/Gas_Source.xlsx
+++ b/data/example/Gas_Source.xlsx
@@ -645,12 +645,12 @@
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>MaxProd</t>
+          <t>GasMaxProd</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>MinProd</t>
+          <t>GasMinProd</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -722,12 +722,12 @@
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>MaxProd</t>
+          <t>GasMaxProd</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>MinProd</t>
+          <t>GasMinProd</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
@@ -795,12 +795,12 @@
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>Maximum active power output of the unit</t>
+          <t>Maximum gas production of gas source</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>Minimum active power output of the unit</t>
+          <t>Minimum gas production of gas source</t>
         </is>
       </c>
       <c r="I5" s="7" t="inlineStr">
@@ -941,12 +941,12 @@
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>[MW]</t>
+          <t>[t/h]</t>
         </is>
       </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>[MW]</t>
+          <t>[t/h]</t>
         </is>
       </c>
       <c r="I7" s="9" t="inlineStr">

</xml_diff>